<commit_message>
Assign HS code 9027900000 to invoice item 5 (Electrode Accessories)
SUP-PH-7001 is a Supmea online pH/ORP meter; pH meters have their own CN
subheading 9027 89 30. The invoice describes the goods as "Accessories for
SUP-PH-7001", so Chapter 90 Note 2(b) classifies them with that instrument.
Note 2(a) does not divert them, since PVC pipe (3917) and bracket/terminal
box cover (3926/7326) are not goods of any heading of Ch. 84, 85, 90 or 91.

=> parts and accessories of heading 9027 = 9027 90 00.

Flag kept as "NAVRH - POTVRDIT": if W.P.E. declares the SUP-PH-7001 itself
as an automatic regulating instrument of heading 9032, the accessories must
follow to 9032900000 instead. Reasoning and the stricter split-by-material
alternative (3917 23 00 + 3926 90 97) documented on the notes sheet.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JVVYVx5LRrePVnb9koUebA
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_WPE_CZ26013054.xlsx
+++ b/output/HS_Code_Summary_WPE_CZ26013054.xlsx
@@ -890,12 +890,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>NUTNO POTVRDIT</t>
+          <t>9027900000</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Příslušenství elektrody pro SUP-PH-7001 – PVC trubky se závitem (1 m), držák trubky, kryt svorkovnice</t>
+          <t>Příslušenství elektrody pro SUP-PH-7001 – PVC trubky se závitem (1 m), držák trubky, kryt svorkovnice; části a příslušenství přístrojů pro fyzikální nebo chemickou analýzu (pH metrů podpoložky 9027 89 30)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -928,12 +928,12 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>K DOŘEŠENÍ</t>
+          <t>NÁVRH – POTVRDIT</t>
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>HS kód NEBYL v e-mailu od S. Hampla uveden (uvedeny jen 8421999090 a 8413502090) ani na B/L. Návrh: 9026909000 / 9027900000 (části a příslušenství měřicích přístrojů) nebo 3917 (plastové trouby). POTVRDIT se zákazníkem před podáním JSD. Hodnota pouze 4,50 EUR.</t>
+          <t>HS kód nebyl uveden v e-mailu ani na B/L. NAVRŽENO 9027900000 = části a příslušenství přístrojů kap. 9027; samotný SUP-PH-7001 (online pH/ORP metr Supmea) patří do 9027 89 30 'pH metry, rH metry'. Pozn. 2 b) ke kap. 90: příslušenství určené výhradně/hlavně pro daný přístroj se zařazuje s tímto přístrojem. ALTERNATIVA: pokud W.P.E. deklaruje SUP-PH-7001 jako regulační/kontrolní přístroj (9032), použít 9032900000. Bez preference (CN). CBAM se nevztahuje. POTVRDIT se zákazníkem.</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Electrode Accessories (4,50 EUR) nemá přidělený HS kód – nutno potvrdit se zákazníkem.</t>
+          <t>Electrode Accessories (4,50 EUR) neměla v podkladech HS kód. NAVRŽENO 9027900000 (části a příslušenství pH metru SUP-PH-7001, podpoložka 9027 89 30). Alternativa 9032900000, pokud je přístroj deklarován jako regulační. Nechat potvrdit zákazníkem – viz list 'Dokumenty a poznámky'.</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>NUTNO POTVRDIT</t>
+          <t>9027900000 (návrh)</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
@@ -1548,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A94"/>
+  <dimension ref="A1:A118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="16">
       <c r="A16" s="18">
-        <f>== ⚠ POLOŽKA 5 – ELECTRODE ACCESSORIES: HS KÓD CHYBÍ ===</f>
+        <f>== ⚠ POLOŽKA 5 – ELECTRODE ACCESSORIES: NÁVRH HS KÓDU 9027900000 ===</f>
         <v/>
       </c>
     </row>
@@ -1665,7 +1665,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tato položka NENÍ pokryta e-mailem (uvedeny pouze 2 HS kódy) ani popisem zboží na B/L.</t>
+          <t>Tato položka NENÍ pokryta e-mailem S. Hampla (uvedeny pouze 2 HS kódy) ani popisem zboží na B/L.</t>
         </is>
       </c>
     </row>
@@ -1677,466 +1677,614 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>→ NUTNO POTVRDIT HS KÓD SE ZÁKAZNÍKEM / SAMUELEM HAMPLEM PŘED PODÁNÍM JSD.</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Možnosti: 9026909000 nebo 9027900000 (části a příslušenství měřicích/kontrolních přístrojů),</t>
+          <t>NAVRŽENÝ KÓD: 9027 90 00 00 (části a příslušenství přístrojů pro fyzikální nebo chemickou analýzu)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   případně 3917 (plastové trouby a hadice). Hodnota je marginální (4,50 EUR), ale položka musí být deklarována.</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Odůvodnění:</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="18">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. SUP-PH-7001 je online pH/ORP metr (transmitter) výrobce Supmea Automation. Pro pH metry existuje</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     vlastní podpoložka KN 9027 89 30 – 'pH metry, rH metry a ostatní přístroje k měření vodivosti'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Faktura zboží výslovně označuje jako 'Accessories for SUP-PH-7001', tj. příslušenství určené</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     výhradně nebo hlavně pro tento konkrétní přístroj.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. Poznámka 2 b) ke kapitole 90: části a příslušenství vhodné pro použití výhradně nebo hlavně</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     s určitým přístrojem se zařazují spolu s tímto druhem přístroje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. Poznámka 2 a) se neuplatní – PVC trubka (3917), držák a kryt svorkovnice (3926/7326) nejsou zbožím</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     žádné položky kapitol 84, 85, 90 ani 91, takže je do vlastní položky 'nevytáhne'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → části a příslušenství přístrojů čísla 9027 = 9027 90 00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA – pokud W.P.E. deklaruje samotný SUP-PH-7001 jako automatický regulační nebo kontrolní</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>přístroj čísla 9032 (přístroj řídí dávkovací čerpadla podle nastavené hodnoty pH), musí příslušenství</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>následovat tento přístroj → 9032 90 00 00. Rozhodnutí přístroj vs. regulátor patří k přístroji samotnému.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>→ DOPORUČENÍ: zeptat se W.P.E. / S. Hampla, pod jakým kódem dováží samotný transmitter SUP-PH-7001,</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   a příslušenství zařadit do odpovídající položky 'části a příslušenství' (9027 90 00 nebo 9032 90 00).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PŘÍSNĚJŠÍ VARIANTA (nedoporučuje se): rozdělit položku podle materiálu – PVC trubky se závitem 3917 23 00,</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>držák a kryt svorkovnice 3926 90 97. Právně obhajitelné, pokud by celní orgán trubky posoudil jako běžnou</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PVC trubku, ale tři sazební položky kvůli 4,50 EUR jsou nepřiměřené; pozn. 2 b) ke kap. 90 hovoří pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ponechání položky pohromadě.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Dopad cla je zanedbatelný (základ 4,67 EUR celní hodnoty), jde o obhajitelnost kódu na JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sazbu cla pro 9027 90 00 ověřit v TARIC k datu propuštění.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="18">
         <f>== ⚠ PREFERENČNÍ PŮVOD (COO) – KONTROLA PROVEDENA ===</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>V žádném z dodaných dokumentů (faktura, packing list, loading info, B/L, telex release) NENÍ preferenční věta.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Deklarovaný původ: Čína – 'Country of origin: China' (faktura i packing list), 'MADE IN CHINA SWM33' (značky, B/L).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>EU nemá s ČLR preferenční dohodu → preferenční sazební zacházení NELZE uplatnit.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>→ Uplatní se PLNÉ třetizemní clo (erga omnes) dle TARIC pro oba HS kódy. Sazbu ověřit v TARIC k datu propuštění.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="18">
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="18">
         <f>== CBAM ===</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>CBAM se na tuto zásilku NEVZTAHUJE.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>HS 8421999090 a 8413502090 spadají do kapitoly 84 (stroje a mechanická zařízení), která NENÍ v příloze I nařízení CBAM.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>CBAM zboží = kapitoly 25 (cement), 28/2804 10 (vodík), 31 (hnojiva), 72/73 (železo a ocel), 76 (hliník), 2716 (elektřina).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>→ Do JSD se kód Y (Y128 / Y238 / Y137 / Y237) neuvádí.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>⚠ UPOZORNĚNÍ K REGISTRU: Příjemce W.P.E. a.s. (Podnikatelská 565, 190 11 Praha) NENÍ uveden</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>v souboru reference/CBAM_receivers_CZ.xlsx (list List1) – ani ve sloupci 'Firma', ani podle EORI,</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>ani mezi firmami mimo EU využívajícími náš sdílený účet CBAM-CZ-2025-QGM67089385721.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Pro tuto zásilku to nevadí (žádné CBAM zboží), ale doporučuji firmu prověřit a doplnit do registru</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>pro případ budoucích zásilek s CBAM zbožím.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="18">
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="18">
         <f>== ANTIDUMPING ===</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>Pro HS 8421999090 (části filtračních/čisticích zařízení) ani 8413502090 (objemová čerpadla s vratným pohybem)</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>s původem v ČLR nebylo antidumpingové opatření zjištěno.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>→ Ověřit v TARIC k datu propuštění (opatření se mění).</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="18">
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="18">
         <f>== OBCHODNÍ SLEVA ===</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Faktura SWM33-260522 NEOBSAHUJE žádnou obchodní slevu. Proporcionální rozpuštění slevy se neuplatní.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="18">
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="18">
         <f>== INCOTERM ===</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>Incoterm: CIF Praha (CIF Prague).</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>Zdroj: faktura, řádek 'CIF Prague port amount €19,079.00'. B/L: FREIGHT PREPAID, port of discharge PRAGUE / PRAHA,</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>final destination PRAGUE / PRAHA. Poznámka na B/L: 'LCL SERVICE CHARGE &amp; DESTINATION CHARGE FOR ACCOUNT OF CNEE'.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>Pozn.: CIF je námořní doložka, ale jmenované místo je vnitrozemská Praha – tak je uvedeno na faktuře.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="18">
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="18">
         <f>== CELNÍ HODNOTA – VÝPOČET ===</f>
         <v/>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>Fakturovaná cena zboží (součet položek 1–5):                     18 383,50 EUR</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>+ Handling cost:                                                       45,50 EUR</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>+ Delivery cost to Shanghai (vnitrozemská přeprava v ČLR):            450,00 EUR</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>+ Shipping freight (námořní přepravné):                               200,00 EUR</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>+ Zaokrouhlení prodejcem:                                               0,50 EUR</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62">
+    <row r="86">
+      <c r="A86">
         <f> CELKEM CIF PRAHA (dle faktury):                                  19 079,00 EUR</f>
         <v/>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>Vedlejší náklady (695,50 EUR) rozpuštěny PROPORCIONÁLNĚ podle hodnoty zboží (faktor 1,0378313).</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="20" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="20" t="inlineStr">
         <is>
           <t>⚠ Součet položek faktury je 19 078,50 EUR, faktura však uvádí celkem 19 079,00 EUR (rozdíl 0,50 EUR –</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t xml:space="preserve">   zaokrouhlení prodejcem, 'SAY EURO NINETEEN THOUSAND SEVENTY-NINE ONLY'). Rozdíl byl rozpuštěn</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t xml:space="preserve">   proporcionálně, aby součet celní hodnoty odpovídal fakturovanému celku 19 079,00 EUR.</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="18">
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="18">
         <f>== ⚠ TÚ 6 824 CZK – NUTNO POTVRDIT ZPŮSOB ZAHRNUTÍ ===</f>
         <v/>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>E-mail S. Hampla uvádí: 'TÚ: 6824 CZK'. Tato částka NENÍ obsažena ve faktuře prodejce.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>Fakturovaná doložka CIF Praha již zahrnuje přepravu až do Prahy, tedy i úsek PO vstupu na celní území EU.</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>Náklady na přepravu po vstupu do EU lze od celní hodnoty odečíst pouze tehdy, jsou-li samostatně vyčísleny –</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>na faktuře prodejce vyčísleny NEJSOU.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="20" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="20" t="inlineStr">
         <is>
           <t>→ POTVRDIT: má se TÚ 6 824 CZK k celní hodnotě PŘIČÍST (dodatečné náklady do místa vstupu do EU),</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t xml:space="preserve">   nebo jde o tuzemský úsek přepravy k ODEČTU? V souhrnu zatím NENÍ zohledněno – celní hodnota je čistě</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t xml:space="preserve">   fakturovaná CIF Praha 19 079,00 EUR.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="18">
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="18">
         <f>== HMOTNOSTI A KOLLI – PŘIŘAZENÍ K HS KÓDŮM ===</f>
         <v/>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>Hmotnosti NEJSOU dopočítávány proporcionálně – packing list i loading info uvádějí hmotnosti přímo po baleních,</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>která se 1:1 kryjí s HS kódy:</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+    <row r="105">
+      <c r="A105" t="inlineStr">
         <is>
           <t xml:space="preserve">   • paleta 1 = položka 1 (MBR membrány)        → 8421999090: 500,0 kg NW / 525,0 kg GW / 50 ks</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
+    <row r="106">
+      <c r="A106" t="inlineStr">
         <is>
           <t xml:space="preserve">   • paleta 2 = položky 2, 3, 4 (dávkovací čerpadla + ND) → 8413502090: 480,0 kg NW / 496,0 kg GW / 28 ks</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
+    <row r="107">
+      <c r="A107" t="inlineStr">
         <is>
           <t xml:space="preserve">   • 2 kartony = položka 5 (příslušenství elektrody)      → HS k potvrzení: 5,0 kg NW / 7,5 kg GW / 9 ks</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
+    <row r="108">
+      <c r="A108" t="inlineStr">
         <is>
           <t>Kontrolní součet: 985,0 kg NW / 1 028,5 kg GW / 87 ks / 4 kolli – souhlasí s PL, loading info i B/L (1 028,500 KGS).</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="18">
+    <row r="109">
+      <c r="A109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="18">
         <f>== KLASIFIKACE PODLE ODESÍLATELE ===</f>
         <v/>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="111">
+      <c r="A111" t="inlineStr">
         <is>
           <t>Zásilka má jediného odesílatele: Hengshui Snowate Environmental Technology Co., Ltd.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="112">
+      <c r="A112" t="inlineStr">
         <is>
           <t>Rozdělení podle odesílatelů se proto neuplatní – všechny řádky patří pod jednoho odesílatele.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="18">
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="18">
         <f>== TERMÍNY ===</f>
         <v/>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
+    <row r="115">
+      <c r="A115" t="inlineStr">
         <is>
           <t>Faktura / packing list:  5. 6. 2026</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
+    <row r="116">
+      <c r="A116" t="inlineStr">
         <is>
           <t>Nakládka:               18. 6. 2026</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
+    <row r="117">
+      <c r="A117" t="inlineStr">
         <is>
           <t>Shipped on board:        3. 7. 2026 (OOCL SWEDEN 008W, Shanghai)</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
+    <row r="118">
+      <c r="A118" t="inlineStr">
         <is>
           <t>Příjezd A1 Praha:       31. 8. 2026</t>
         </is>

</xml_diff>